<commit_message>
Full update: All 13 Regions Screenshot and Excel
</commit_message>
<xml_diff>
--- a/weather_history.xlsx
+++ b/weather_history.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>Βροχόπτωση</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Περιφέρεια</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,6 +486,7 @@
           <t>Μ/Δ</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -508,6 +514,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -535,6 +542,7 @@
           <t>Μ/Δ</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -562,6 +570,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -589,6 +598,7 @@
           <t>Μ/Δ</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -616,6 +626,7 @@
           <t>Μ/Δ</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -643,6 +654,7 @@
           <t>Μ/Δ</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -670,6 +682,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -697,6 +710,7 @@
           <t>Μ/Δ</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -724,6 +738,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -751,6 +766,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -778,6 +794,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -805,6 +822,7 @@
           <t>0.2</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -832,6 +850,7 @@
           <t>0.0</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -857,6 +876,3079 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>0.0</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Αίγινα</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ελευσίνα</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ελληνικό</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Κοτρώνι</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Λαύριο</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Μαρκόπουλο</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Μέγαρα</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Νέα Φιλαδέλφεια Αυτόματος</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>18.7</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ο.Α.Κ.Α.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ολυμπιακό Κολυμβητήριο</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>18.7</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ραφήνα</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>16.7</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Σπάτα Αεροδρόμιο</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Σχοινιάς</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>17.7</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Τατόι</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>17.9</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ψυτάλεια</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>19.5</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>11.0</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Attiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Αλεξανδρούπολη</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Δράμα</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Θάσος</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Καβάλα</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ξάνθη</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ορμένιο</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Σουφλί</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>East_Macedonia_and_Thrace</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Έδεσσα</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>17.5</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Central_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Θεσσαλονίκη</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>15.8</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Central_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Πολύκαστρο</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17.7</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Central_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Σέρρες</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Central_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Καστοριά</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>West_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Κοζάνη</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>West_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Φλώρινα</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>17.2</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>West_Macedonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Άκτιο</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>8.9</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Epirus</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Ιωάννινα</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Epirus</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Κόνιτσα</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Epirus</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Αγχίαλος</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Thessaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Κρανέα</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>15.6</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Thessaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Λάρισα</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Thessaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Σκιάθος</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Thessaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Σοφάδες</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Thessaly</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Αργοστόλι</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Ionian_Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Ζάκυνθος</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Ionian_Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Κέρκυρα</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Ionian_Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Οθωνοί</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Ionian_Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Στροφάδες</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Ionian_Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Ανδραβίδα</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>West_Greece</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Αντίρριο</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15.9</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>West_Greece</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Άραξος</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>17.3</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>West_Greece</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Κυλλήνη</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>West_Greece</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Μεσολόγγι</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>West_Greece</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Δεσφίνα</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>17.9</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Κάρυστος</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Κάτω Τιθορέα</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>21.2</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Κύμη</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Λαμία</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>19.9</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Σκύρος</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Τανάγρα</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>18.6</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Ωρεοί</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>18.8</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Sterea</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Αντικύθηρα</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>18.3</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Άργος (Πυργέλα)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Καλαμάτα</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Κύθηρα</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Κύθηρα Πόλη</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Λεωνίδιο</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>9.2</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Μεθώνη</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Τρίπολη</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>17.8</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>-0.3</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Peloponnese</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Άγιος Ευστράτιος</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Ικαρία</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Λήμνος</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>16.2</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Μυτιλήνη</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Σάμος</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>16.8</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Χίος</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>17.0</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Ψαρά</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>North_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Αστυπάλαια</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17.8</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Κάλυμνος</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Κάρπαθος</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>18.7</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>13.8</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Κάσος</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Καστελόριζο</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Κύθνος</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>17.1</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>11.8</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Κως</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>17.4</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Λέρος</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>17.8</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>13.9</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Μήλος</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Μήλος Αεροδρόμιο</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Μύκονος</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>17.0</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Νάξος</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Νάξος Πόλη</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Πάρος</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>17.2</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Ρόδος</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>19.6</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>12.6</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Σαντορίνη</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Σύρος</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>17.0</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Τήνος</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>South_Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Γαύδος</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Ηράκλειο</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>17.8</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Ιεράπετρα</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Καστέλι Πεδιάδος</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>16.7</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Παλαιόχωρα</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Σητεία</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Σούδα Χανιά</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Τυμπάκι</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Μ/Δ</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Crete</t>
         </is>
       </c>
     </row>

</xml_diff>